<commit_message>
Update CAFIRA Excel: add owner names, products, B2B/B2C classification
Removed stand, Instagram, address, and rubro columns. Added:
- Contact names (owners/founders) found via web research for ~20 companies
- "Qué venden" column with specific product descriptions
- B2B/B2C/Ambos classification for each exhibitor

https://claude.ai/code/session_01MygzCe54Ft5eDHcYzUExQQ
</commit_message>
<xml_diff>
--- a/Expositores_CAFIRA_2026.xlsx
+++ b/Expositores_CAFIRA_2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Expositores CAFIRA 2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Expositores CAFIRA 2026'!$A$1:$I$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Expositores CAFIRA 2026'!$A$1:$G$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,18 +439,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,42 +459,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Stand</t>
+          <t>Teléfono / WhatsApp</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Teléfono / WhatsApp</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Sitio Web</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Sitio Web</t>
+          <t>Contacto (Dueño/Gerente)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>Qué venden</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Contacto (Dueño/Gerente)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Rubro</t>
+          <t>B2B / B2C</t>
         </is>
       </c>
     </row>
@@ -508,38 +496,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>1166092892</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1166092892</t>
+          <t>ventas@tiendadecostumbres.com.ar</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ventas@tiendadecostumbres.com.ar</t>
+          <t>www.tiendadecostumbres.com.ar</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>www.tiendadecostumbres.com.ar</t>
+          <t>Silvina Lippai (Fundadora)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>@tiendadecostumbres</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Regina Pacini de Alvear 892, Don Torcuato</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Alfombras, Textil Hogar</t>
+          <t>Alfombras, almohadones y pies de cama tejidos 100% a mano con lana de oveja y llama</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -551,36 +533,34 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>11 5320-2300</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>11 5320-2300</t>
+          <t>hello.omaobjetos@gmail.com</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>hello.omaobjetos@gmail.com</t>
+          <t>www.omaobjetos.com.ar</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>www.omaobjetos.com.ar</t>
+          <t>María (Fundadora)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>@oma_objetos</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Coronel Pringles 1645</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
+          <t>Objetos de diseño artesanal, iluminación y aromatización para el hogar</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -590,36 +570,30 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>+54 9 11 5420-0863</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 5420-0863</t>
+          <t>alcarpintero@yahoo.com.ar</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>alcarpintero@yahoo.com.ar</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
           <t>alcarpintero.com.ar</t>
         </is>
       </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>@alcarpintero</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Humberto Primo 1919, Avellaneda (CP1870), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
+          <t>Muebles y objetos de carpintería artística en madera</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -629,36 +603,34 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>11 7227 1001</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>11 7227 1001</t>
+          <t>info@makiwarmi</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>info@makiwarmi</t>
+          <t>www.makiwarmi.com</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>www.makiwarmi.com</t>
+          <t>Glenda Saintotte (Fundadora)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>@maki_warmi</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>España 837, San Isidro</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+          <t>Alfombras artesanales de lana tejidas a mano por tejedoras del norte argentino</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -668,36 +640,30 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>11 3506 4003</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>11 3506 4003</t>
+          <t>rnunez@casanunez.com.ar</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>rnunez@casanunez.com.ar</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
           <t>www.casanunez.com.ar</t>
         </is>
       </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>@casanunez</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Av. Gaona 4280, Moreno / Av. San Martín 3502, CABA</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+          <t>Muebles de exterior y jardín en materiales resistentes a la intemperie</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>B2C</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -707,24 +673,26 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>KM 44</t>
+          <t>+54 9 11 3166 3868</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 3166 3868</t>
+          <t>blossommarket@hotmail.com</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>KM 44 Paseo Pilar Shopping Del Viso</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Decoración mayorista para el hogar</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -732,26 +700,20 @@
           <t>Ganeshas</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>223</t>
-        </is>
-      </c>
+      <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>@ganeshas.argentinas</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Av. Agustín M. García 8765, Nordelta</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>Objetos de decoración</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -761,34 +723,28 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>3512373016</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>3512373016</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
           <t>casamanica.deco@gmail.com</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Sofía Simes</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>@casamanica</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>9 de julio 3286, Córdoba (CP5000)</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Alfombras, Objetos Deco</t>
+          <t>Alfombras turcas y objetos de decoración</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -800,38 +756,28 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>1126730866</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1126730866</t>
+          <t>disegnoprimo@gmail.com</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>disegnoprimo@gmail.com</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>disegnoprimo.com.ar</t>
         </is>
       </c>
+      <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>@Disegnoprimo</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Cita previa, Don Torcuato (CP1611), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Hierro</t>
+          <t>Objetos de diseño en hierro para decoración</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -843,28 +789,34 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>(+5411) 5272-5140</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>(+5411) 5272-5140</t>
+          <t>info@baitpisos.com.ar</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>info@baitpisos.com.ar</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Fitz Roy 2179, CABA</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+          <t>baitpisos.com.ar</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Diego Joel Fleisman (Dueño)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Pisos, revestimientos, griferías, sanitarios y artículos de decoración</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -874,38 +826,28 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>4981-4564 / +54 9 11 4430-1750</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>4981-4564 / +54 9 11 4430-1750</t>
+          <t>bonndeco@gmail.com</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>bonndeco@gmail.com</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>bonndecomayorista.com</t>
         </is>
       </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>@bonndeco_</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Pasaje King 356, CABA (CP1199)</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Cuadros y Espejos, Objetos Deco</t>
+          <t>Espejos biselados y cuadros decorativos (mayorista)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -917,38 +859,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>+54 9 2494 63-2550 / +54 9 2494 24-8474</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>+54 9 2494 63-2550 / +54 9 2494 24-8474</t>
+          <t>oxidopampastandil@gmail.com</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>oxidopampastandil@gmail.com</t>
+          <t>oxidopampas.com</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>oxidopampas.com</t>
+          <t>Marcos Probicito, Carolina Liernur, Gonzalo Juárez (Fundadores)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>@oxidopampasmayorista</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Parque Industrial, Calle 116 e/111 y 113, Tandil (CP7000)</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Hierro, Macetas y Jardín, Objetos Deco</t>
+          <t>Fogones, asadores, parrillas y accesorios en hierro oxidado</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -960,38 +896,28 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>01173738716</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>01173738716</t>
+          <t>rhiedeco@gmail.com</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>rhiedeco@gmail.com</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
           <t>rhie.com.ar</t>
         </is>
       </c>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>@rhieobjetos</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Avenida Centenario 1528, Beccar (CP1643)</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Velas y Esencias</t>
+          <t>Velas, esencias y objetos de decoración artesanal</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1003,34 +929,28 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>11 21828720</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>11 21828720</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
           <t>alma.dusha@hotmail.com</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Silvana y Leo (Fundadores)</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>@alma_dusha</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Acceso Oeste y Camino del Buen Ayre, Moreno (CP1742)</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco</t>
+          <t>Objetos decorativos de chapa y hierro artesanales</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1042,38 +962,32 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>+54 9 1147780491</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1147780491</t>
+          <t>ventas@bigbudahome.com.ar</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ventas@bigbudahome.com.ar</t>
+          <t>www.bgbgift.com.ar</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>www.bgbgift.com.ar</t>
+          <t>Federico y María Eugenia (Fundadores)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>@reinabatatamayorista</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Godoy Cruz 1457, CABA (C1414CYE)</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Bazar, Objetos Deco</t>
+          <t>Bazar boutique, objetos de decoración y regalería</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1085,36 +999,30 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>5493412243484</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>5493412243484</t>
+          <t>ventas@plugiluminacion.com.ar</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ventas@plugiluminacion.com.ar</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
           <t>plugiluminacion.com.ar</t>
         </is>
       </c>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>@plugiluminacion</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Asamblea 420, Rosario (CP2000), Santa Fe</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
+          <t>Luminarias y artículos de iluminación</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1124,32 +1032,26 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>01150641144</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>01150641144</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
           <t>hedan.decor@gmail.com</t>
         </is>
       </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>@HEDAN.decor</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Hudson (CP1885), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
+          <t>Objetos de decoración</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1157,22 +1059,20 @@
           <t>Bosco</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>271</t>
-        </is>
-      </c>
+      <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>@boscoargentina</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
+          <t>Decoración para el hogar</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1182,36 +1082,30 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>1131742347</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1131742347</t>
+          <t>info@gcfdesign.com.ar</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>info@gcfdesign.com.ar</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
           <t>www.gcfdesign.com.ar</t>
         </is>
       </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>@Gcfdesign</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Av. Corrientes 4006, piso 1 Of. 2, Almagro</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr"/>
+          <t>Empapelados decorativos y vinilos de diseño</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1221,38 +1115,28 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>1162829914</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1162829914</t>
+          <t>Aurorahouse.ar@gmail.com</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Aurorahouse.ar@gmail.com</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
           <t>www.aurorahouse.com.ar</t>
         </is>
       </c>
+      <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>@aurorahouse.ar</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires 1398, Tigre (1648)</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación</t>
+          <t>Lámparas de macramé y hierro con diseños exclusivos</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1264,36 +1148,34 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>4584-5953 / 5491156388499</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>4584-5953 / 5491156388499</t>
+          <t>info@component-newhouse.com</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>info@component-newhouse.com</t>
+          <t>www.component-newhouse.com</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>www.component-newhouse.com</t>
+          <t>Pablo Rafael Pelletieri (Socio)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>@component_yz</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Almirante Francisco Segui 2469, CABA (CP1416)</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr"/>
+          <t>Muebles de diseño</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1303,38 +1185,28 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>2215700991</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>2215700991</t>
+          <t>soyhebras@gmail.com</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>soyhebras@gmail.com</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
           <t>hebrastejido.mitiendanube.com</t>
         </is>
       </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>@hebras_handmade</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Soler 107, Chascomús (CP7130), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación</t>
+          <t>Lámparas y objetos tejidos artesanales</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1346,38 +1218,28 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>01169952113</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>01169952113</t>
+          <t>ventas@alchemystba.com</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ventas@alchemystba.com</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
           <t>www.alchemystba.com.ar</t>
         </is>
       </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>@alchemystba</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Araoz 2437, Palermo, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Empapelados, Textil Hogar</t>
+          <t>Murales y empapelados de autor, textiles para el hogar</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1389,36 +1251,34 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>+54 341 4432731</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+54 341 4432731</t>
+          <t>info@pasionariaargentina.com.ar</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>info@pasionariaargentina.com.ar</t>
+          <t>www.pasionariaargentina.com.ar</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>www.pasionariaargentina.com.ar</t>
+          <t>Carina Cavazza y Mario Gerosa (Fundadores / CEO)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>@lapasionariaargentina</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Av. Eva Perón 8960, Rosario</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr"/>
+          <t>Cosmética, perfumería, velas de soja y difusores para el hogar</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1428,34 +1288,28 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>03513890157</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>03513890157</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
           <t>pachi54@hotmail.com</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Pachi Grosso</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>@Pachi_decohome</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Av. Los Álamos 1111 La Rufina CP 5151, La Calera, Córdoba</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Textil Hogar</t>
+          <t>Textiles artesanales en lana de oveja del norte argentino</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1467,32 +1321,30 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>+54 91150130162</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+54 91150130162</t>
+          <t>hola@thestampa.com.ar</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>hola@thestampa.com.ar</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
           <t>www.thestampa.com.ar</t>
         </is>
       </c>
+      <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>@thestampa</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
+          <t>Cuadros y láminas decorativas</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1502,34 +1354,28 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>277</t>
+          <t>11 4523-3711 / 54 9 1139157987</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>11 4523-3711 / 54 9 1139157987</t>
+          <t>clientes@midekocollection.com.ar</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>clientes@midekocollection.com.ar</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
           <t>midekocollection.com.ar</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Bucarelli 1162, CABA (CP1427)</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco</t>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Objetos de decoración y regalería importada (mayorista)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -1541,38 +1387,28 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>+54 9 11 2874-7827</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 2874-7827</t>
+          <t>proveedores@aldealobos.com.ar</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>proveedores@aldealobos.com.ar</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
           <t>aldealobos.com.ar</t>
         </is>
       </c>
+      <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>@aldea.lobos</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Argerich 1480, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación, Objetos Deco</t>
+          <t>Iluminación y objetos decorativos (fabricante mayorista)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -1584,34 +1420,24 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>+54 9 1134803734</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1134803734</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
           <t>eukenedeco@gmail.com</t>
         </is>
       </c>
+      <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>@Eukenedeco</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Parque Leloir, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Flores</t>
+          <t>Flores artificiales y arreglos decorativos</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1623,38 +1449,28 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>3515905832</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>3515905832</t>
+          <t>mbaconsultas@gmail.com</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>mbaconsultas@gmail.com</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
           <t>mbaaprons.mitiendanube.com</t>
         </is>
       </c>
+      <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>@mba_aprons</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Angualasto 7522, Villa Warcalde, Córdoba</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Textil Hogar</t>
+          <t>Delantales y textiles para el hogar</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1666,34 +1482,24 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>159</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
           <t>11 25 99 83 72</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>sincreticodeco.mitiendanube.com</t>
         </is>
       </c>
+      <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>@sincreticodeco</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Galería Libertad – Libertad 1170, local 23</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Textil Hogar</t>
+          <t>Alfombras, mantas, almohadones artesanales de comunidades indígenas (economía solidaria)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1705,38 +1511,28 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>+54 9 3516156817</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>+54 9 3516156817</t>
+          <t>abrilhomedeco@gmail.com</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>abrilhomedeco@gmail.com</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
           <t>abrildeco.com</t>
         </is>
       </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>@abrilhomedeco</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Av. Rafael Núñez 4565, Córdoba (CP5009)</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco, Plantas y Flores</t>
+          <t>Macetas rotomoldeadas de diseño, muebles de ratán y objetos deco</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1748,34 +1544,28 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>2664154064</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2664154064</t>
+          <t>administracion@valdense.com.ar</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>administracion@valdense.com.ar</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
           <t>www.valdense.com.ar</t>
         </is>
       </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>@evelynhome&amp;deco</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Rieles</t>
+          <t>Rieles de aluminio y accesorios para cortinas</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -1787,36 +1577,30 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>+541161233189</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>+541161233189</t>
+          <t>info@mekkhome.com.ar</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>info@mekkhome.com.ar</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
           <t>mekkmayorista.com.ar</t>
         </is>
       </c>
+      <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>@mekk.home</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>San Isidro, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr"/>
+          <t>Objetos de decoración y hogar importados (mayorista)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1826,34 +1610,24 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>+54-11-6125-5635 / +54-11-5009-5455</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>+54-11-6125-5635 / +54-11-5009-5455</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
           <t>ventas@avcinteriores.com.ar</t>
         </is>
       </c>
+      <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>@avc.interiores</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Muebles, Sillones</t>
+          <t>Sofás, sillones y muebles para living, comedor y exterior</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -1865,38 +1639,28 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>+54 9 1150152542</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1150152542</t>
+          <t>info@alamada.com.ar</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>info@alamada.com.ar</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
           <t>alamada.com.ar</t>
         </is>
       </c>
+      <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>@casa.alamada</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Ruiz Huidobro 2783, CP 1429 CABA</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>Muebles, Objetos Deco</t>
+          <t>Muebles y accesorios decorativos de diseño</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1908,38 +1672,28 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>+54 9 2915439953</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>+54 9 2915439953</t>
+          <t>mavacuadros@yahoo.com.ar</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>mavacuadros@yahoo.com.ar</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
           <t>mavacuadros.com.ar</t>
         </is>
       </c>
+      <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>@mavacuadros</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Bahía Blanca (CP8000), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Cuadros y Espejos</t>
+          <t>Cuadros, marcos y espejos artesanales</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1951,38 +1705,28 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>1127952502</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1127952502</t>
+          <t>teodorashome@gmail.com</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>teodorashome@gmail.com</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
           <t>teodoranordelta.mitiendanube.com</t>
         </is>
       </c>
+      <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>@teodorashome</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Talcahuano 1201 CP 1014, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>Blanquería, Textil Hogar</t>
+          <t>Blanquería y textiles para el hogar</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -1994,38 +1738,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>+54 9 1165052654</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1165052654</t>
+          <t>maraniadeco@gmail.com</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>maraniadeco@gmail.com</t>
+          <t>Marania.com.ar</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Marania.com.ar</t>
+          <t>Alicita Morea, Belén y Bernardi (Fundadoras)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>@maraniadeco</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Recoleta, CABA</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación</t>
+          <t>Lámparas artesanales, apliques, candelabros y objetos de iluminación hechos a mano</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2037,38 +1775,28 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>+54 9 3562 56-5475</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>+54 9 3562 56-5475</t>
+          <t>chapitadeco@gmail.com</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>chapitadeco@gmail.com</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
           <t>chapitadeco.com.ar</t>
         </is>
       </c>
+      <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>@chapitadeco</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>España 387 CP 2421, Morteros, Córdoba</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco</t>
+          <t>Maceteros, portamacetas, fogoneros y figuras en chapa oxidada</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2080,42 +1808,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>+54 9 4572-3954 / +54 9 1144981805</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>+54 9 4572-3954 / +54 9 1144981805</t>
+          <t>alinahegi@yahoo.com</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>alinahegi@yahoo.com</t>
+          <t>alinahegi.com</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>alinahegi.com</t>
+          <t>Alina Hegi (Dueña)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>@alinahegi</t>
+          <t>Muebles de diseño y objetos decorativos</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Alina Hegi</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>Manuela Pedraza 6064, CP 1431, CABA</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Muebles, Objetos Deco</t>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2127,36 +1845,30 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>+54 9 1146278813 / +54 9 1152282166</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1146278813 / +54 9 1152282166</t>
+          <t>ventas@nikeliluminacion.com.ar</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>ventas@nikeliluminacion.com.ar</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
           <t>Nikeliluminacion.com.ar</t>
         </is>
       </c>
+      <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>@Nikeliluminacionok</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Mons Angelelli 936 CP 1708, Morón, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr"/>
+          <t>Luminarias decorativas de diseño y fabricación propia</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2166,38 +1878,28 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>+5491136916804</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>+5491136916804</t>
+          <t>colombas.sp@gmail.com</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>colombas.sp@gmail.com</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
           <t>Colombas.com.ar</t>
         </is>
       </c>
+      <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>@colombas_buenos_aires</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco, Textil Hogar</t>
+          <t>Objetos de decoración y textiles para el hogar</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2209,38 +1911,28 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>+54 9 1138651657 / +54 9 1142105434</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1138651657 / +54 9 1142105434</t>
+          <t>petrishome2@gmail.com</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>petrishome2@gmail.com</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
           <t>Petris.com.ar</t>
         </is>
       </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>@petris.home</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>José A. Blanco 4238, CP 1879, Quilmes, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>Bazar</t>
+          <t>Bazar y artículos para el hogar</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2252,38 +1944,32 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>03482412015</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>03482412015</t>
+          <t>hola@allegrahome.com.ar</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>hola@allegrahome.com.ar</t>
+          <t>allegrahome.com.ar</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>allegrahome.com.ar</t>
+          <t>Carolina y Mauro (Fundadores)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>@allegrahome</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Roca 944, Reconquista CP 3560, Santa Fe</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco, Textil Hogar</t>
+          <t>Mantelería de algodón antimanchas, regalería textil y objetos deco</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2295,34 +1981,24 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>+54 9 1151634000</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1151634000</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
           <t>decocontemporary@gmail.com</t>
         </is>
       </c>
+      <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>@contemporarydeco</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>Calle del Caminante 80, apt 250, Nordelta (CP1670)</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>Bazar</t>
+          <t>Bazar y artículos decorativos</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2334,34 +2010,28 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>3525509346</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>3525509346</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
           <t>lucasmsilva75@gmail.com</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Lucas M. Silva (Dueño)</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>@silvaandco.ar</t>
+          <t>Iluminación, muebles y objetos de decoración</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Lucas M. Silva</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación, Muebles, Objetos Deco</t>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2373,38 +2043,28 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>+54 9 1142023905 / +54 9 1143996590</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1142023905 / +54 9 1143996590</t>
+          <t>info@alhambra.com.ar</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>info@alhambra.com.ar</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
           <t>alhambra.com.ar</t>
         </is>
       </c>
+      <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>@alhambra.telas</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>Gral. Villegas 1071, Remedios de Escalada (CP1826)</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>Textil Hogar</t>
+          <t>Telas para decoración y tapicería (distribuidora mayorista, +50 años)</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -2416,38 +2076,32 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>3518733702 / 3515932694</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>3518733702 / 3515932694</t>
+          <t>marhaba.homeargentina@gmail.com</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>marhaba.homeargentina@gmail.com</t>
+          <t>marhabacarpets.com</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>marhabacarpets.com</t>
+          <t>Federica Fontana y Esteban (Fundadores) / Rodo y Rochi (Socios Argentina)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>@marhaba_carpets</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>Av Japón 2300, Córdoba</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>Textil Hogar</t>
+          <t>Alfombras orientales, persas, de yute, algodón y lino</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2459,34 +2113,24 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>+54 9 1166337427</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1166337427</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
           <t>decocraft@hotmail.com</t>
         </is>
       </c>
+      <c r="D51" s="2" t="inlineStr"/>
       <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>@craft_dec2</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Itaqui 2182, CABA</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación</t>
+          <t>Lámparas y objetos de iluminación artesanal</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2498,38 +2142,28 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>+549 1162966000</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>+549 1162966000</t>
+          <t>broderidesign@gmail.com</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>broderidesign@gmail.com</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
           <t>broderi.com.ar</t>
         </is>
       </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>@broderi.manteles</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>Entre Rios 2056, Olivos (CP1636), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>Bazar, Platería</t>
+          <t>Manteles, caminos de mesa, artículos de bazar y platería</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2541,38 +2175,32 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>+54 9 11 45883857 / +54 9 1158423499</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 45883857 / +54 9 1158423499</t>
+          <t>administracion@e-bony.com.ar</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>administracion@e-bony.com.ar</t>
+          <t>e-bony.com.ar</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>e-bony.com.ar</t>
+          <t>Lionel Elias Steisel (Gerente)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>@ebonymueblesok</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Paysandu 1451 CP 1416 CABA</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>Muebles</t>
+          <t>Muebles clásicos artesanales tallados en cedro y roble</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2584,34 +2212,24 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>+54 9 11 2280 7278</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 2280 7278</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
           <t>botanybuenosaires@gmail.com</t>
         </is>
       </c>
+      <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>@Botany.bsas</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>Quilmes, Buenos Aires (CP1879)</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>Velas y Esencias</t>
+          <t>Velas y esencias aromáticas</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2623,34 +2241,28 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>4855-1212 / +54 9 1136929553</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>4855-1212 / +54 9 1136929553</t>
+          <t>info@datetux.com.ar</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>info@datetux.com.ar</t>
+          <t>datelux.com.ar</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>@Dateluxok</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>Scalabrini Ortiz 250, CP 1414, CABA</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación</t>
+          <t>Artefactos de iluminación importados y componentes</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2662,38 +2274,28 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>+54 9 1130092394</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1130092394</t>
+          <t>byfelideco.tienda@gmail.com</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>byfelideco.tienda@gmail.com</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
           <t>linktr.ee/By_felideco</t>
         </is>
       </c>
+      <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>@byfelideco</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>CABA</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco, Textil Hogar</t>
+          <t>Objetos de decoración y textiles para el hogar</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2705,38 +2307,28 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>+54 9 1138097211 / +54 9 1123721176</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1138097211 / +54 9 1123721176</t>
+          <t>loladecoarg@gmail.com</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>loladecoarg@gmail.com</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
           <t>lola-deco.negocio.site</t>
         </is>
       </c>
+      <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>@loladecoarg</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>El Talar CP 1617, Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>Sillones</t>
+          <t>Sillones y muebles tapizados a medida</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2748,38 +2340,28 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>45525055 / +54 9 1155843078</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>45525055 / +54 9 1155843078</t>
+          <t>miradorobjetos@gmail.com</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>miradorobjetos@gmail.com</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
           <t>mirador.com.ar</t>
         </is>
       </c>
+      <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>@miradorporelmundo</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>Giribone 1960, CABA (CP1427)</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco</t>
+          <t>Muebles y objetos importados en madera, ratán y fibras naturales (mayorista)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -2791,38 +2373,28 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>+54 9 1151857964</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1151857964</t>
+          <t>info@lederhd.com</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>info@lederhd.com</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
           <t>lederhd.com</t>
         </is>
       </c>
+      <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>@Leder_hd</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>Av. Libertador 13821, Martínez, Buenos Aires (CP1640)</t>
-        </is>
-      </c>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>Alfombras, Muebles, Objetos Deco, Sillones</t>
+          <t>Muebles, alfombras, sillones y marroquinería en cuero artesanal (desde 1927)</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2834,38 +2406,28 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>+54 9 1147710073 / +54 9 11 3167-4471</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1147710073 / +54 9 11 3167-4471</t>
+          <t>consultas@desdeasia.com.ar</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>consultas@desdeasia.com.ar</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
           <t>desdeasia.com</t>
         </is>
       </c>
+      <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>@desde_asia</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>Malabia 1359, Palermo (CP1414), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>Muebles, Objetos Deco</t>
+          <t>Muebles y objetos decorativos orientales importados de Asia</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2877,38 +2439,28 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>+54 9 11 64486916 / +54 9 11 42284886</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 64486916 / +54 9 11 42284886</t>
+          <t>info@cuerosespeciales.com</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>info@cuerosespeciales.com</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
           <t>cuerosespeciales.com</t>
         </is>
       </c>
+      <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>@cueros_especiales</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>Pte. Perón 3145, Valentín Alsina / Av. Hipólito Yrigoyen 6602, Lanús</t>
-        </is>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>Sillones</t>
+          <t>Sillones, sillas, almohadones y alfombras en cuero (fabricante desde 1986)</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2920,38 +2472,28 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>+54 9 1124712225</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1124712225</t>
+          <t>info@cadmia.com.ar</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>info@cadmia.com.ar</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
           <t>cadmia.com.ar</t>
         </is>
       </c>
+      <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>@cadmiahome</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>Juncal 1115, CABA (1062)</t>
-        </is>
-      </c>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>Textil Hogar</t>
+          <t>Textiles de diseño estampados a mano para el hogar</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -2963,38 +2505,32 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>+54 9 3472 532010</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>+54 9 3472 532010</t>
+          <t>Hola@estilodomingo.com.ar</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Hola@estilodomingo.com.ar</t>
+          <t>estilodomingo.com.ar</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>estilodomingo.com.ar</t>
+          <t>Matías y Ayelén (Fundadores, arquitectos)</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>@estilo.domingo</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>Córdoba</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco</t>
+          <t>Objetos de decoración en madera (maceteros, espejos, lámparas, +120 productos)</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -3006,38 +2542,32 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>+54 9 3516312332 / +54 9 3515936034</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>+54 9 3516312332 / +54 9 3515936034</t>
+          <t>Iameclectica@gmail.com</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Iameclectica@gmail.com</t>
+          <t>eclecticadiseno.com.ar</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>eclecticadiseno.com.ar</t>
+          <t>Emilia, Eugenia y Mariangeles Alexandroff Zlateff (Fundadoras)</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>@eclectica.diseno</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>Doctor Orlando Severo Melone 250, Córdoba (CP5000)</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>Objetos Deco</t>
+          <t>Objetos de diseño en madera y cuero para hogar y gastronomía</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -3049,38 +2579,28 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>+54 9 2215736756</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>+54 9 2215736756</t>
+          <t>Fabivaioli@gmail.com</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Fabivaioli@gmail.com</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
           <t>casiunangeldeco.mitiendanube.com</t>
         </is>
       </c>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>@Casiunangel_deco</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>Calle 77 n°1886, La Plata (CP1900), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>Borlas</t>
+          <t>Borlas decorativas y accesorios textiles</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -3092,34 +2612,24 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>+54 9 1163677970</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1163677970</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
           <t>mrc_sofa@hotmail.com</t>
         </is>
       </c>
+      <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>@fabricaar</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>Martin Peschel 600, Tres de Febrero (CP1657), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>Sillones</t>
+          <t>Sillones y sofás tapizados</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -3131,38 +2641,28 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>+54 9 11 64331266 / +54 9 1164055659</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 64331266 / +54 9 1164055659</t>
+          <t>info@forevents.com.ar</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>info@forevents.com.ar</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
           <t>Forevents.com.ar</t>
         </is>
       </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>@Forevents_</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr"/>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>Hipólito Yrigoyen 1764, Garín (CP1619), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>Muebles, Sillas, Sillones</t>
+          <t>Muebles, sillas Tiffany y mobiliario para eventos</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>B2B</t>
         </is>
       </c>
     </row>
@@ -3174,34 +2674,24 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>3564 508778</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>3564 508778</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
           <t>galponmuebles@gmail.com</t>
         </is>
       </c>
+      <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>@Galponmuebles</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Calle 9, Frontera (CP2348), Santa Fe</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>Muebles, Sillas, Sillones</t>
+          <t>Muebles, sillas y sillones</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -3213,38 +2703,32 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>275</t>
+          <t>+54 9 11 62446973 / +54 9 1130684132</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>+54 9 11 62446973 / +54 9 1130684132</t>
+          <t>Lampsilver@gmail.com</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Lampsilver@gmail.com</t>
+          <t>Lampsilver.com.ar</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Lampsilver.com.ar</t>
+          <t>Santiago Maldonado (Fundador)</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>@Lampsilver</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>Ayacucho 662, Florida – Vte Lopez (CP1642), Buenos Aires</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Iluminación</t>
+          <t>Lámparas artísticas y de diseño artesanal</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
@@ -3256,43 +2740,33 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>+54 9 1135914398</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>+54 9 1135914398</t>
+          <t>Ortigacasa.ar@gmail.com</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Ortigacasa.ar@gmail.com</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
           <t>Ortiga.com.ar</t>
         </is>
       </c>
+      <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>@Ortigacasa</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>CABA</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>Vajilla</t>
+          <t>Vajilla y artículos de mesa</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I70"/>
+  <autoFilter ref="A1:G70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 3 more contact names from web research (total 23/69)
Found via web search: René García (Petris), Victoria Williams Becker
(Cadmia), Maryan y Jeru (Teodoras Home). Remaining 46 companies don't
publish owner names publicly.

https://claude.ai/code/session_01MygzCe54Ft5eDHcYzUExQQ
</commit_message>
<xml_diff>
--- a/Expositores_CAFIRA_2026.xlsx
+++ b/Expositores_CAFIRA_2026.xlsx
@@ -1718,10 +1718,14 @@
           <t>teodoranordelta.mitiendanube.com</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Maryan y Jeru (Fundadoras)</t>
+        </is>
+      </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Blanquería y textiles para el hogar</t>
+          <t>Blanquería, diseño de interiores y muebles a medida</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -1924,10 +1928,14 @@
           <t>Petris.com.ar</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>René García (Dueño)</t>
+        </is>
+      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Bazar y artículos para el hogar</t>
+          <t>Vajilla y objetos de cerámica artesanal para el hogar</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -2485,7 +2493,11 @@
           <t>cadmia.com.ar</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Victoria Williams Becker (Fundadora)</t>
+        </is>
+      </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
           <t>Textiles de diseño estampados a mano para el hogar</t>

</xml_diff>